<commit_message>
Nome vira o campo chave e nome fantasia vira razao social
O campo obrigatorio passa a se chamar apenas Nome (e e por ele que a
importacao casa as linhas). O segundo campo guarda a razao social, o nome do
contrato: a coluna trade_name foi renomeada para legal_name para o banco dizer
o que guarda.

No importador, "Razao Social" deixou de ser apelido da coluna de nome e virou
coluna propria — antes uma planilha com as duas colunas importaria a razao
social como se fosse o nome da conta.

Co-authored-by: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modelo_Importacao_Leadrix_CRM.xlsx
+++ b/Modelo_Importacao_Leadrix_CRM.xlsx
@@ -399,28 +399,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:U4"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="21.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="26.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
-    <col min="15" max="15" width="31.83203125" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
-    <col min="17" max="17" width="21.83203125" customWidth="1"/>
-    <col min="18" max="18" width="22.83203125" customWidth="1"/>
-    <col min="19" max="19" width="24.83203125" customWidth="1"/>
-    <col min="20" max="20" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="21.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="31.83203125" customWidth="1"/>
+    <col min="17" max="17" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="21.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="24.83203125" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,60 +429,63 @@
         <v>Cliente</v>
       </c>
       <c r="B1" t="str">
+        <v>Razão social</v>
+      </c>
+      <c r="C1" t="str">
         <v>CNPJ</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Site</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Classificação</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Mercado</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Microssegmento</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Porte</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Nível ABM</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Campanha</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Termômetro</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Canal de origem</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Origem do lead</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Origem (especificar)</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Quem indicou</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Comissão de indicação (%)</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Contato (Nome)</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Contato (Cargo)</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Contato (E-mail)</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Contato (Telefone)</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Observações</v>
       </c>
     </row>
@@ -490,60 +494,63 @@
         <v>Metalúrgica Serra Azul</v>
       </c>
       <c r="B2" t="str">
+        <v>Serra Azul Indústria Metalúrgica S.A.</v>
+      </c>
+      <c r="C2" t="str">
         <v>11.222.333/0001-81</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>www.serraazul.ind.br</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Conta-alvo</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Indústria</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Metalmecânica e autopeças</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Grande</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>1:1</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>IA no fluxo real da operação</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>60</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Prospecção ativa (ABM)</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Boomit</v>
       </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
       <c r="N2" t="str">
         <v/>
       </c>
-      <c r="O2">
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2">
         <v>10</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>Carlos Mendes</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>Diretor de Operações</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v>carlos.mendes@serraazul.ind.br</v>
       </c>
-      <c r="S2" t="str">
+      <c r="T2" t="str">
         <v>+55 11 98888-1111</v>
       </c>
-      <c r="T2" t="str">
+      <c r="U2" t="str">
         <v>Trocou de ERP em 2026; processos administrativos ainda em planilha.</v>
       </c>
     </row>
@@ -594,18 +601,21 @@
         <v/>
       </c>
       <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v>Luiza Faria</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>Gerente de TI</v>
       </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
         <v>luiza.faria@serraazul.ind.br</v>
       </c>
-      <c r="S3" t="str">
-        <v/>
-      </c>
       <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
         <v/>
       </c>
     </row>
@@ -614,73 +624,76 @@
         <v>Vértice Consultoria Empresarial</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Vértice Consultoria Empresarial Ltda.</v>
       </c>
       <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
         <v>www.vertice.com.br</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Cliente</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Serviços B2B</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Consultorias</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Média</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>1:few</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>Crescer sem ampliar a estrutura na mesma proporção</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>75</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>Indicação</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>Outros</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>Parceiro de tecnologia</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>Ana Prado (evento Febraban)</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>5</v>
       </c>
-      <c r="P4" t="str">
+      <c r="Q4" t="str">
         <v>Ricardo Souza</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>Sócio</v>
       </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
         <v>ricardo@vertice.com.br</v>
       </c>
-      <c r="S4" t="str">
+      <c r="T4" t="str">
         <v>+55 41 96666-3333</v>
       </c>
-      <c r="T4" t="str">
+      <c r="U4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -707,108 +720,116 @@
         <v>Obrigatório</v>
       </c>
       <c r="B3" t="str">
-        <v>Só a coluna "Cliente". Todo o resto é opcional.</v>
+        <v>Só a coluna "Cliente" (o nome pelo qual o time chama a conta). Todo o resto é opcional.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Uma conta por nome</v>
+        <v>Nome x Razão social</v>
       </c>
       <c r="B4" t="str">
-        <v>Linhas com o mesmo nome de conta são agrupadas. Use uma linha por contato e repita só o nome.</v>
+        <v>O nome é a chave da importação; a razão social é o nome do contrato e não participa do casamento.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nome é a chave</v>
+        <v>Uma conta por nome</v>
       </c>
       <c r="B5" t="str">
-        <v>A importação casa pelo NOME (ignorando maiúsculas). Nome existente é atualizado; nome novo cria conta. "Acme" e "Acme Brasil" viram duas contas — padronize antes.</v>
+        <v>Linhas com o mesmo nome de conta são agrupadas. Use uma linha por contato e repita só o nome.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Célula vazia não apaga</v>
+        <v>Nome é a chave</v>
       </c>
       <c r="B6" t="str">
-        <v>Reimportar não zera o que já está preenchido no CRM: só sobrescreve o que vier preenchido na planilha.</v>
+        <v>A importação casa pelo NOME (ignorando maiúsculas). Nome existente é atualizado; nome novo cria conta. "Acme" e "Acme Brasil" viram duas contas — padronize antes.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Dado fora do padrão</v>
+        <v>Célula vazia não apaga</v>
       </c>
       <c r="B7" t="str">
-        <v>Não é gravado: o campo fica vazio e a linha aparece no quadro de avisos da tela, com o número da linha da planilha.</v>
+        <v>Reimportar não zera o que já está preenchido no CRM: só sobrescreve o que vier preenchido na planilha.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CNPJ e e-mail</v>
+        <v>Dado fora do padrão</v>
       </c>
       <c r="B8" t="str">
-        <v>São validados. Inválidos não entram e geram aviso; o resto da linha é importado normalmente.</v>
+        <v>Não é gravado: o campo fica vazio e a linha aparece no quadro de avisos da tela, com o número da linha da planilha.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Cargo do contato</v>
+        <v>CNPJ e e-mail</v>
       </c>
       <c r="B9" t="str">
-        <v>Vale preencher: é o que monta o mapa do grupo decisor (patrocinador, operações, TI, financeiro, jurídico).</v>
+        <v>São validados. Inválidos não entram e geram aviso; o resto da linha é importado normalmente.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Comissão</v>
+        <v>Cargo do contato</v>
       </c>
       <c r="B10" t="str">
-        <v>Informe o número do percentual (10 = 10%). Em branco, a conta fica sem comissão de indicação.</v>
+        <v>Vale preencher: é o que monta o mapa do grupo decisor (patrocinador, operações, TI, financeiro, jurídico).</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Origem "Outros"</v>
+        <v>Comissão</v>
       </c>
       <c r="B11" t="str">
-        <v>Exige a coluna "Origem (especificar)" preenchida.</v>
+        <v>Informe o número do percentual (10 = 10%). Em branco, a conta fica sem comissão de indicação.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Colunas</v>
+        <v>Origem "Outros"</v>
       </c>
       <c r="B12" t="str">
-        <v>A ordem não importa e colunas desconhecidas são ignoradas. Pode apagar as colunas que não usar.</v>
+        <v>Exige a coluna "Origem (especificar)" preenchida.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>Colunas</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>A ordem não importa e colunas desconhecidas são ignoradas. Pode apagar as colunas que não usar.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Onde importar</v>
+        <v/>
       </c>
       <c r="B14" t="str">
-        <v>CRM → Importador → selecione o arquivo → confira a pré-visualização e os avisos → Importar.</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>Onde importar</v>
+      </c>
+      <c r="B15" t="str">
+        <v>CRM → Importador → selecione o arquivo → confira a pré-visualização e os avisos → Importar.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
         <v>Formatos</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B16" t="str">
         <v>XLSX, XLS ou CSV (UTF-8).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Quinto mercado: Outros, com especificacao obrigatoria
A conta que nao se encaixa nos quatro mercados do site precisava entrar
na base de alguma forma. Em vez de forcar um mercado errado, agora existe
"Outros (especificar)": o setor real vai num campo de texto proprio, e
tanto o formulario quanto o banco recusam salvar sem ele, para a
categoria nao virar um balaio sem informacao.

As dores e indicadores de Outros sao os genericos da Leadrix (margem,
capacidade, qualidade, risco, receita) — nao ha especificidade inventada
de um setor que nao foi estudado. Prioridade ABM "seletiva".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modelo_Importacao_Leadrix_CRM.xlsx
+++ b/Modelo_Importacao_Leadrix_CRM.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:V4"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -407,21 +407,22 @@
     <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="19.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="21.83203125" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="26.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="31.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="21.83203125" customWidth="1"/>
-    <col min="19" max="19" width="22.83203125" customWidth="1"/>
-    <col min="20" max="20" width="24.83203125" customWidth="1"/>
-    <col min="21" max="21" width="17.83203125" customWidth="1"/>
+    <col min="7" max="7" width="27.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="21.83203125" customWidth="1"/>
+    <col min="14" max="14" width="20.83203125" customWidth="1"/>
+    <col min="15" max="15" width="26.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="31.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
+    <col min="19" max="19" width="21.83203125" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
+    <col min="21" max="21" width="24.83203125" customWidth="1"/>
+    <col min="22" max="22" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,48 +445,51 @@
         <v>Mercado</v>
       </c>
       <c r="G1" t="str">
+        <v>Mercado (especificar)</v>
+      </c>
+      <c r="H1" t="str">
         <v>Microssegmento</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Porte</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Nível ABM</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Campanha</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Termômetro</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Canal de origem</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Origem do lead</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Origem (especificar)</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Quem indicou</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Comissão de indicação (%)</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Contato (Nome)</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Contato (Cargo)</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Contato (E-mail)</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Contato (Telefone)</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Observações</v>
       </c>
     </row>
@@ -508,49 +512,49 @@
       <c r="F2" t="str">
         <v>Indústria</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Metalmecânica e autopeças</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Grande</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>1:1</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>IA no fluxo real da operação</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>60</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Prospecção ativa (ABM)</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Boomit</v>
       </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
       <c r="O2" t="str">
         <v/>
       </c>
-      <c r="P2">
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2">
         <v>10</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>Carlos Mendes</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v>Diretor de Operações</v>
       </c>
-      <c r="S2" t="str">
+      <c r="T2" t="str">
         <v>carlos.mendes@serraazul.ind.br</v>
       </c>
-      <c r="T2" t="str">
+      <c r="U2" t="str">
         <v>+55 11 98888-1111</v>
       </c>
-      <c r="U2" t="str">
+      <c r="V2" t="str">
         <v>Trocou de ERP em 2026; processos administrativos ainda em planilha.</v>
       </c>
     </row>
@@ -573,9 +577,6 @@
       <c r="F3" t="str">
         <v/>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
@@ -604,18 +605,21 @@
         <v/>
       </c>
       <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
         <v>Luiza Faria</v>
       </c>
-      <c r="R3" t="str">
+      <c r="S3" t="str">
         <v>Gerente de TI</v>
       </c>
-      <c r="S3" t="str">
+      <c r="T3" t="str">
         <v>luiza.faria@serraazul.ind.br</v>
       </c>
-      <c r="T3" t="str">
-        <v/>
-      </c>
       <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
         <v/>
       </c>
     </row>
@@ -638,62 +642,62 @@
       <c r="F4" t="str">
         <v>Serviços B2B</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Consultorias</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Média</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>1:few</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>Crescer sem ampliar a estrutura na mesma proporção</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>75</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>Indicação</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>Outros</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>Parceiro de tecnologia</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>Ana Prado (evento Febraban)</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>5</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>Ricardo Souza</v>
       </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
         <v>Sócio</v>
       </c>
-      <c r="S4" t="str">
+      <c r="T4" t="str">
         <v>ricardo@vertice.com.br</v>
       </c>
-      <c r="T4" t="str">
+      <c r="U4" t="str">
         <v>+55 41 96666-3333</v>
       </c>
-      <c r="U4" t="str">
+      <c r="V4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -797,39 +801,47 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Colunas</v>
+        <v>Mercado "Outros"</v>
       </c>
       <c r="B13" t="str">
-        <v>A ordem não importa e colunas desconhecidas são ignoradas. Pode apagar as colunas que não usar.</v>
+        <v>Exige a coluna "Mercado (especificar)" com o setor da conta.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>Colunas</v>
       </c>
       <c r="B14" t="str">
-        <v/>
+        <v>A ordem não importa e colunas desconhecidas são ignoradas. Pode apagar as colunas que não usar.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Onde importar</v>
+        <v/>
       </c>
       <c r="B15" t="str">
-        <v>CRM → Importador → selecione o arquivo → confira a pré-visualização e os avisos → Importar.</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>Onde importar</v>
+      </c>
+      <c r="B16" t="str">
+        <v>CRM → Importador → selecione o arquivo → confira a pré-visualização e os avisos → Importar.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>Formatos</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B17" t="str">
         <v>XLSX, XLS ou CSV (UTF-8).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -863,7 +875,7 @@
         <v>Mercado</v>
       </c>
       <c r="B3" t="str">
-        <v>Serviços B2B · Indústria · Varejo e Franquias · Empresas Digitais</v>
+        <v>Serviços B2B · Indústria · Varejo e Franquias · Empresas Digitais · Outros (especificar)</v>
       </c>
     </row>
     <row r="4">
@@ -871,7 +883,7 @@
         <v>Microssegmento</v>
       </c>
       <c r="B4" t="str">
-        <v>Texto livre, mas use a lista de Configurações. Ex.: Consultorias · Alimentos e bebidas · Supermercados e varejo alimentar · SaaS B2B</v>
+        <v xml:space="preserve">Texto livre, mas use a lista de Configurações. Ex.: Consultorias · Alimentos e bebidas · Supermercados e varejo alimentar · SaaS B2B · </v>
       </c>
     </row>
     <row r="5">

</xml_diff>